<commit_message>
Uploaded the Correct video into the github repo
</commit_message>
<xml_diff>
--- a/Milestone_2_Resources/F4C_Opossum_6748_Orbital_Project_Logs.xlsx
+++ b/Milestone_2_Resources/F4C_Opossum_6748_Orbital_Project_Logs.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Ld7CK8uqEd2mw9kBftLj+xQGVKAHcLshTKv4KplYu0Y="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="7ydu5UmtkZlKr8nBhYxpB9faRnFrd3qKHYzoNtPzZUA="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="116">
   <si>
     <t>S/N</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Created slides and recorded a video of what we want to achieve in this Orbital Project</t>
+  </si>
+  <si>
+    <t>MILESTONE 1 TRACKING</t>
   </si>
   <si>
     <t>Unity project setup and scene configuration 
@@ -220,6 +223,349 @@
   </si>
   <si>
     <t>Writing of Milestone 1 README documentation</t>
+  </si>
+  <si>
+    <t>MILESTONE 2 TRACKING</t>
+  </si>
+  <si>
+    <t>Sourcing cohesive 2D assets and environment sprites</t>
+  </si>
+  <si>
+    <t>Scoured itch.io, Kenney.nl, and Unity Asset Store for free-to-use 2D assets. Spent a massive amount of time finding character sprites and background layers that actually shared a cohesive pixel-art style so the game wouldn't look like a mismatched patchwork.</t>
+  </si>
+  <si>
+    <t>Overall testing and looking at how the game mode should flow</t>
+  </si>
+  <si>
+    <t>Reading through the scripts currently written and looking for ways to utilise them for the creation of new character and enemy sprites</t>
+  </si>
+  <si>
+    <t>Making sure that any new changes by creating new sprites can utilise scripts that are already written in the earlier milestone stage</t>
+  </si>
+  <si>
+    <t>Trying out new sprites with unique sprite renders to see how the unit progresses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- </t>
+  </si>
+  <si>
+    <t>Build the first character that is using a different image, i.e. the unit image instead of a circle</t>
+  </si>
+  <si>
+    <t>Fixing GitHub Repo merge conflict (1)</t>
+  </si>
+  <si>
+    <t>First Github repo conflict where my partner did the project without syncing to github (did manually zip), and did a push force wiping out all the past history commits. Had to manually restore the git history on my end and add in his edited code to make the current process seemless</t>
+  </si>
+  <si>
+    <t>Adding another sprite to see how different sprites units intereact with one another</t>
+  </si>
+  <si>
+    <t>Testing to see the collison scripts in unit move still work and there is no issues there even if they are different sprite renders</t>
+  </si>
+  <si>
+    <t>Fixing GitHub Repo merge conflict (2)</t>
+  </si>
+  <si>
+    <t>After fixing the main branch, my partner was still working on his version side, i.e. to say was unable to do git pull so essentially the lack of legecy issue along with the new additional commits again required to repeat the whole process again. At least it is not as bad this time around as a github branch was created this time, so the main branch was unaffected</t>
+  </si>
+  <si>
+    <t>Standardizing Sprite PPU and Pivot Points</t>
+  </si>
+  <si>
+    <t>Noticed units were spawning at drastically different scales and floating above the ground. Standardized the Pixel Per Unit (PPU) settings across all imported art assets and manually realigned the center anchor points in the Unity Sprite Editor.</t>
+  </si>
+  <si>
+    <t>Animator Controller Setup &amp; State Machines</t>
+  </si>
+  <si>
+    <t>Built the complex visual State Machines for all new unit types. Mapped out transition conditions (IsMoving, AttackTrig) and spent hours debugging the "Has Exit Time" issue where units would wait for an animation to finish before attacking.</t>
+  </si>
+  <si>
+    <t>Implementing Animation Events for Combat</t>
+  </si>
+  <si>
+    <t>Transitioned damage calculation from a procedural timer to Unity Animation Events. Configured the ExecuteAttack() method to trigger on the exact frame the sword connects in the animation timeline, making combat feel much more responsive.</t>
+  </si>
+  <si>
+    <t>Engineering the CancelAttack Interrupt State</t>
+  </si>
+  <si>
+    <t>Discovered a bug where units got stuck in an attack loop if their target died mid-swing. Engineered an emergency interrupt trigger (CancelAttack) in the Animator State Machine to force units back to an idle state immediately.</t>
+  </si>
+  <si>
+    <t>Economy Backend Logic &amp; Observer Pattern</t>
+  </si>
+  <si>
+    <t>Built the backend logic for passive Gold generation and EXP tracking. Decoupled the UI from the game state using the Observer Pattern so that the UI only updates when an economy event is broadcasted, preventing unnecessary per-frame UI rendering.</t>
+  </si>
+  <si>
+    <t>UI Refactoring: Dynamic Unit Spawning Costs</t>
+  </si>
+  <si>
+    <t>Updated the SpawnUnitFromUI script. Instead of hardcoding buttons, passed a unitIndex parameter to dynamically check if the player has enough gold based on the unitCosts array before instantiating the prefab.</t>
+  </si>
+  <si>
+    <t>Advanced Unit Formation and Movement Animation</t>
+  </si>
+  <si>
+    <t>Refined the UnitMove script so that it accommodates different units speeds to ensure no animation jittering and unrealistic stop-start behaviour would occur.</t>
+  </si>
+  <si>
+    <t>Fixing GitHub Repo merge conflict (3)</t>
+  </si>
+  <si>
+    <t>Partner forgot to do a git pull and change the branch he was working on, so I needed to redo the manual merging again</t>
+  </si>
+  <si>
+    <t>Main Menu Development and Overall Environmental Polish</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>Building the following features:
+1) The layout of the Main Menu (finding the assets, needing to crop the assest, resizing, using photopea for image editing)</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve"> [10 hours]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">2) The scripts for animation of the backdroup, the parllex effect, the unit animations </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">[2 hours] 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">3) Setting up the Canvas for the UI buttons and title, as well as the transition animations between scenes </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">[3 hours]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">4) Adding Splash Screen to the Unity build, to make it more presonalised, as well as using a custom template for the index.html file to host the game </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>[1 hour]</t>
+    </r>
+  </si>
+  <si>
+    <t>Music and Sound Effects System</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">1) Finding free online audio music for gameplay, main menu screen, SFX </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">[2 hours]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">2) Integrating background music, button hover effects, click sound and making persisitent audio management using managers, as well as creating volume slides to change audio level </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>[6 hours]</t>
+    </r>
+  </si>
+  <si>
+    <t>User Interface Refinement and Asset Integration</t>
+  </si>
+  <si>
+    <t>Updated the gameplay UI screen to make it look nicer with images/boards that match the theme we are going for. Had to do some AI generation images since we were unable to find many good images online for free</t>
+  </si>
+  <si>
+    <t>Implementing a Pause Menu</t>
+  </si>
+  <si>
+    <t>Allow for game mode pause if the user wants to stop the game, where audio settings changes are also available, and if the user wants to go back to main menu he / she is able to do so</t>
+  </si>
+  <si>
+    <t>Turret construction and defence system interaction</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>1) Finding / Generating turret and base assets so that they complement one another, making sure the turret has idle and attack animations. Had to manually scrape/edit to obtain each picture needed for turret and base</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve"> [6 hours]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>2) Updating the UI for the castle base (new collision box and moving spawn points), adding buttons for UI to build "scaffolding" to house the turret, as well as buttons to purchase the turret</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve"> [3 hours]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">3) Creating and debugging animation scripts for the turret idle and attack animations, need to time the frame as much as I can based on the images we had </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>[2 hours]</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t>3) Creating scripts for turret projection, where the arrow can come in an arc format since the crossbow has an image animation that shoots slightly upwards, so we want to make the projectile like a "honing missile" with an arc</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Times New Roman"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="12.0"/>
+      </rPr>
+      <t xml:space="preserve"> [5 hours]</t>
+    </r>
+  </si>
+  <si>
+    <t>Overall gameplay testing, debugging and final polishing</t>
+  </si>
+  <si>
+    <t>While we do test each feature each time we implement it, this test is a totallty of all the test we had done from milestone 1 to milestone 2, inlcuding one final test run on how the game should flow.</t>
+  </si>
+  <si>
+    <t>Poster preparation / design for Milestone 2</t>
+  </si>
+  <si>
+    <t>Created a new poster based on the new requirements, which is A1 size. Also spent quite some time finding/generating assets like icons to make the poster look cleaner</t>
+  </si>
+  <si>
+    <t>Milestone 2 Video Production &amp; Editing</t>
+  </si>
+  <si>
+    <t>Looking through all our documentation to create content required for the milestone 2 video submission. Recorded gameplay footage showcasing the new systems and dynamic collision tracking. Recording voiceover explanations going through our progress for milestone 2</t>
+  </si>
+  <si>
+    <t>ReadME documentation update to include Milestone 2</t>
+  </si>
+  <si>
+    <t>Added in the parts that I had designed / created into the read me documentation, as well as finding/creating the scenarios for the images inside the doucmentation</t>
+  </si>
+  <si>
+    <t>Updating Project Logs for Milestone 2</t>
   </si>
   <si>
     <t>TOTAL HOURS WORKED</t>
@@ -235,7 +581,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -254,8 +600,19 @@
       <name val="Times New Roman"/>
     </font>
     <font/>
+    <font>
+      <b/>
+      <sz val="12.0"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -270,12 +627,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFDBE9F7"/>
         <bgColor rgb="FFDBE9F7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border/>
     <border>
       <left style="thin">
@@ -313,11 +676,41 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -334,14 +727,31 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -686,334 +1096,324 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="8" ht="25.5" customHeight="1">
+      <c r="A8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3">
-        <v>46165.0</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3">
+        <v>46165.0</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" s="3">
-        <v>46167.0</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="3">
         <v>46167.0</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="2">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="3">
+        <v>46167.0</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C11" s="3">
-        <v>46168.0</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2">
-        <v>9.0</v>
+        <v>8.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="3">
         <v>46168.0</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E12" s="2">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" s="3">
-        <v>46169.0</v>
-      </c>
-      <c r="D13" s="2" t="s">
+        <v>46168.0</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="2">
         <v>2.0</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3">
         <v>46169.0</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="2">
         <v>2.0</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G14" s="6"/>
+        <v>27</v>
+      </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="3">
+        <v>46169.0</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="3">
-        <v>46170.0</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="E15" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G15" s="6"/>
+      <c r="G15" s="10"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" s="3">
         <v>46170.0</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>11</v>
+      <c r="D16" s="2">
+        <v>1.0</v>
       </c>
       <c r="E16" s="2">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>32</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G16" s="10"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2">
-        <v>14.0</v>
+        <v>13.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" s="3">
         <v>46170.0</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="2">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C18" s="3">
         <v>46170.0</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E18" s="2">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="3">
+        <v>46170.0</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="C19" s="3">
-        <v>46171.0</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" s="3">
-        <v>46172.0</v>
-      </c>
-      <c r="D20" s="2" t="s">
+        <v>46171.0</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E20" s="2">
         <v>2.0</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="2">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="3">
         <v>46172.0</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="2">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="2">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="3">
+        <v>46172.0</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="C22" s="3">
-        <v>46173.0</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="2">
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C23" s="3">
         <v>46173.0</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="2">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="2">
-        <v>21.0</v>
+        <v>20.0</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" s="3">
         <v>46173.0</v>
@@ -1022,18 +1422,18 @@
         <v>11</v>
       </c>
       <c r="E24" s="2">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="2">
-        <v>22.0</v>
+        <v>21.0</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C25" s="3">
         <v>46173.0</v>
@@ -1042,18 +1442,18 @@
         <v>11</v>
       </c>
       <c r="E25" s="2">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="2">
-        <v>23.0</v>
+        <v>22.0</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C26" s="3">
         <v>46173.0</v>
@@ -1062,163 +1462,714 @@
         <v>11</v>
       </c>
       <c r="E26" s="2">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="3">
+        <v>46173.0</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25" customHeight="1">
+      <c r="A28" s="9">
         <v>24.0</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="3">
-        <v>46174.0</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="F27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="28" ht="14.25" customHeight="1">
-      <c r="A28" s="2">
-        <v>25.0</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="C28" s="3">
         <v>46174.0</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E28" s="2">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25" customHeight="1">
+      <c r="A29" s="9">
+        <v>25.0</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="29" ht="14.25" customHeight="1">
-      <c r="A29" s="2">
-        <v>26.0</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="C29" s="3">
         <v>46174.0</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="2">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="F29" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" ht="14.25" customHeight="1">
+      <c r="A30" s="9">
+        <v>26.0</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="30" ht="14.25" customHeight="1">
-      <c r="A30" s="2">
-        <v>27.0</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="C30" s="3">
         <v>46174.0</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="2">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="F30" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" ht="14.25" customHeight="1">
+      <c r="A31" s="9">
+        <v>27.0</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="31" ht="14.25" customHeight="1">
-      <c r="A31" s="2">
-        <v>28.0</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="C31" s="3">
         <v>46174.0</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="9">
+        <v>1.0</v>
+      </c>
+      <c r="E31" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" ht="14.25" customHeight="1">
+      <c r="A32" s="9">
+        <v>28.0</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="3">
+        <v>46174.0</v>
+      </c>
+      <c r="D32" s="9">
         <v>3.0</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E32" s="9">
         <v>3.0</v>
       </c>
-      <c r="F31" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="32" ht="14.25" customHeight="1">
-      <c r="A32" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="F32" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="9">
+    </row>
+    <row r="33" ht="25.5" customHeight="1">
+      <c r="A33" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9">
+        <v>29.0</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="3">
         <v>46174.0</v>
       </c>
-      <c r="D32" s="8">
-        <f>SUM($D$2:$D31)</f>
-        <v>11</v>
-      </c>
-      <c r="E32" s="8">
-        <f>SUM($E$2:$E31)</f>
+      <c r="D34" s="9">
+        <v>10.0</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G34" s="9"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="12"/>
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12"/>
+      <c r="T34" s="12"/>
+      <c r="U34" s="12"/>
+      <c r="V34" s="12"/>
+      <c r="W34" s="12"/>
+      <c r="X34" s="12"/>
+      <c r="Y34" s="12"/>
+      <c r="Z34" s="12"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9">
+        <v>30.0</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="3">
+        <v>46174.0</v>
+      </c>
+      <c r="D35" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9">
+        <v>31.0</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="3">
+        <v>46174.0</v>
+      </c>
+      <c r="D36" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9">
+        <v>32.0</v>
+      </c>
+      <c r="B37" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="F32" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
+      <c r="C37" s="13">
+        <v>46175.0</v>
+      </c>
+      <c r="D37" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9">
+        <v>33.0</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" s="13">
+        <v>46176.0</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9">
+        <v>34.0</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="13">
+        <v>46177.0</v>
+      </c>
+      <c r="D39" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9">
+        <v>35.0</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="13">
+        <v>46178.0</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9">
+        <v>36.0</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="D41" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9">
+        <v>37.0</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C42" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="D42" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9">
+        <v>38.0</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43" s="13">
+        <v>46180.0</v>
+      </c>
+      <c r="D43" s="9">
+        <v>12.0</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9">
+        <v>39.0</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C44" s="13">
+        <v>46181.0</v>
+      </c>
+      <c r="D44" s="9">
+        <v>10.0</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9">
+        <v>40.0</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C45" s="13">
+        <v>46183.0</v>
+      </c>
+      <c r="D45" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9">
+        <v>41.0</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C46" s="13">
+        <v>46185.0</v>
+      </c>
+      <c r="D46" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9">
+        <v>42.0</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="13">
+        <v>46187.0</v>
+      </c>
+      <c r="D47" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9">
+        <v>43.0</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C48" s="13">
+        <v>46188.0</v>
+      </c>
+      <c r="D48" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="E48" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9">
+        <v>44.0</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C49" s="13">
+        <v>46193.0</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="50" ht="149.25" customHeight="1">
+      <c r="A50" s="14">
+        <v>45.0</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" s="13">
+        <v>46195.0</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="14">
+        <v>15.0</v>
+      </c>
+      <c r="F50" s="14" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51" ht="149.25" customHeight="1">
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="13">
+        <v>46197.0</v>
+      </c>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9">
+        <v>46.0</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C52" s="13">
+        <v>46197.0</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9">
+        <v>47.0</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C53" s="13">
+        <v>46198.0</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9">
+        <v>48.0</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C54" s="13">
+        <v>46199.0</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9">
+        <v>49.0</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C55" s="13">
+        <v>46200.0</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="9">
+        <v>16.0</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9">
+        <v>50.0</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C56" s="13">
+        <v>46201.0</v>
+      </c>
+      <c r="D56" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="E56" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9">
+        <v>51.0</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C57" s="13">
+        <v>46201.0</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9">
+        <v>52.0</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C58" s="13">
+        <v>46202.0</v>
+      </c>
+      <c r="D58" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9">
+        <v>53.0</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C59" s="13">
+        <v>46202.0</v>
+      </c>
+      <c r="D59" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="E59" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="60" ht="38.25" customHeight="1">
+      <c r="A60" s="9">
+        <v>54.0</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C60" s="13">
+        <v>46202.0</v>
+      </c>
+      <c r="D60" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="E60" s="9">
+        <v>2.0</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="61" ht="14.25" customHeight="1">
+      <c r="A61" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B61" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C61" s="16">
+        <v>46174.0</v>
+      </c>
+      <c r="D61" s="15">
+        <f t="array" ref="D61">SUM($D$2:INDEX(D:D, ROW()-1))</f>
+        <v>106</v>
+      </c>
+      <c r="E61" s="15">
+        <f t="array" ref="E61">SUM($E$2:INDEX(E:E, ROW()-1))</f>
+        <v>158</v>
+      </c>
+      <c r="F61" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
     <row r="62" ht="14.25" customHeight="1"/>
     <row r="63" ht="14.25" customHeight="1"/>
     <row r="64" ht="14.25" customHeight="1"/>
@@ -2158,10 +3109,47 @@
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="1001" ht="14.25" customHeight="1"/>
+    <row r="1002" ht="14.25" customHeight="1"/>
+    <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
+    <row r="1005" ht="14.25" customHeight="1"/>
+    <row r="1006" ht="14.25" customHeight="1"/>
+    <row r="1007" ht="14.25" customHeight="1"/>
+    <row r="1008" ht="14.25" customHeight="1"/>
+    <row r="1009" ht="14.25" customHeight="1"/>
+    <row r="1010" ht="14.25" customHeight="1"/>
+    <row r="1011" ht="14.25" customHeight="1"/>
+    <row r="1012" ht="14.25" customHeight="1"/>
+    <row r="1013" ht="14.25" customHeight="1"/>
+    <row r="1014" ht="14.25" customHeight="1"/>
+    <row r="1015" ht="14.25" customHeight="1"/>
+    <row r="1016" ht="14.25" customHeight="1"/>
+    <row r="1017" ht="14.25" customHeight="1"/>
+    <row r="1018" ht="14.25" customHeight="1"/>
+    <row r="1019" ht="14.25" customHeight="1"/>
+    <row r="1020" ht="14.25" customHeight="1"/>
+    <row r="1021" ht="14.25" customHeight="1"/>
+    <row r="1022" ht="14.25" customHeight="1"/>
+    <row r="1023" ht="14.25" customHeight="1"/>
+    <row r="1024" ht="14.25" customHeight="1"/>
+    <row r="1025" ht="14.25" customHeight="1"/>
+    <row r="1026" ht="14.25" customHeight="1"/>
+    <row r="1027" ht="14.25" customHeight="1"/>
+    <row r="1028" ht="14.25" customHeight="1"/>
+    <row r="1029" ht="14.25" customHeight="1"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="17">
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F50:F51"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="D4:D5"/>
@@ -2169,7 +3157,6 @@
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="F6:F7"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>